<commit_message>
added features in inventory
</commit_message>
<xml_diff>
--- a/NAP FORM 1 (FORMAT).xlsx
+++ b/NAP FORM 1 (FORMAT).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Employee Records Management System\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C40372C6-B6E5-43F5-8581-55D8A26714D4}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FA420D3-F22D-494A-A0D0-8ECD8F011647}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DE8C5812-6A99-445C-91C0-D3EC6F6B46CC}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="45">
   <si>
     <t>1. NAME OF OFFICE:</t>
   </si>
@@ -217,6 +217,15 @@
   </si>
   <si>
     <t>Name</t>
+  </si>
+  <si>
+    <t>Sub Category</t>
+  </si>
+  <si>
+    <t>Entry</t>
+  </si>
+  <si>
+    <t>CATEGORY</t>
   </si>
 </sst>
 </file>
@@ -913,6 +922,159 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="6"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -937,163 +1099,10 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2290,97 +2299,97 @@
       <c r="C3" s="5"/>
       <c r="D3" s="6"/>
       <c r="E3" s="7"/>
-      <c r="F3" s="108" t="s">
+      <c r="F3" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="G3" s="109"/>
-      <c r="H3" s="109"/>
-      <c r="I3" s="110"/>
-      <c r="J3" s="108" t="s">
+      <c r="G3" s="68"/>
+      <c r="H3" s="68"/>
+      <c r="I3" s="69"/>
+      <c r="J3" s="67" t="s">
         <v>1</v>
       </c>
-      <c r="K3" s="109"/>
-      <c r="L3" s="109"/>
-      <c r="M3" s="109"/>
-      <c r="N3" s="111" t="s">
+      <c r="K3" s="68"/>
+      <c r="L3" s="68"/>
+      <c r="M3" s="68"/>
+      <c r="N3" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="O3" s="112"/>
-      <c r="P3" s="113"/>
+      <c r="O3" s="71"/>
+      <c r="P3" s="72"/>
     </row>
     <row r="4" spans="1:16" ht="25.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="E4" s="9"/>
-      <c r="F4" s="114" t="s">
+      <c r="F4" s="73" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="115"/>
-      <c r="H4" s="115"/>
-      <c r="I4" s="116"/>
-      <c r="J4" s="120" t="s">
+      <c r="G4" s="74"/>
+      <c r="H4" s="74"/>
+      <c r="I4" s="75"/>
+      <c r="J4" s="79" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="121"/>
-      <c r="L4" s="121"/>
-      <c r="M4" s="121"/>
-      <c r="N4" s="117"/>
-      <c r="O4" s="118"/>
-      <c r="P4" s="122"/>
+      <c r="K4" s="80"/>
+      <c r="L4" s="80"/>
+      <c r="M4" s="80"/>
+      <c r="N4" s="76"/>
+      <c r="O4" s="77"/>
+      <c r="P4" s="81"/>
     </row>
     <row r="5" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="E5" s="9"/>
-      <c r="F5" s="114"/>
-      <c r="G5" s="115"/>
-      <c r="H5" s="115"/>
-      <c r="I5" s="116"/>
-      <c r="J5" s="101" t="s">
+      <c r="F5" s="73"/>
+      <c r="G5" s="74"/>
+      <c r="H5" s="74"/>
+      <c r="I5" s="75"/>
+      <c r="J5" s="82" t="s">
         <v>5</v>
       </c>
-      <c r="K5" s="102"/>
-      <c r="L5" s="102"/>
-      <c r="M5" s="102"/>
-      <c r="N5" s="101" t="s">
+      <c r="K5" s="83"/>
+      <c r="L5" s="83"/>
+      <c r="M5" s="83"/>
+      <c r="N5" s="82" t="s">
         <v>6</v>
       </c>
-      <c r="O5" s="102"/>
-      <c r="P5" s="103"/>
+      <c r="O5" s="83"/>
+      <c r="P5" s="84"/>
     </row>
     <row r="6" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="E6" s="9"/>
-      <c r="F6" s="117"/>
-      <c r="G6" s="118"/>
-      <c r="H6" s="118"/>
-      <c r="I6" s="119"/>
-      <c r="J6" s="123"/>
-      <c r="K6" s="124"/>
-      <c r="L6" s="124"/>
-      <c r="M6" s="124"/>
-      <c r="N6" s="125"/>
-      <c r="O6" s="118"/>
-      <c r="P6" s="122"/>
+      <c r="F6" s="76"/>
+      <c r="G6" s="77"/>
+      <c r="H6" s="77"/>
+      <c r="I6" s="78"/>
+      <c r="J6" s="85"/>
+      <c r="K6" s="86"/>
+      <c r="L6" s="86"/>
+      <c r="M6" s="86"/>
+      <c r="N6" s="87"/>
+      <c r="O6" s="77"/>
+      <c r="P6" s="81"/>
     </row>
     <row r="7" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="E7" s="9"/>
-      <c r="F7" s="98" t="s">
+      <c r="F7" s="88" t="s">
         <v>7</v>
       </c>
-      <c r="G7" s="99"/>
-      <c r="H7" s="99"/>
-      <c r="I7" s="100"/>
-      <c r="J7" s="98" t="s">
+      <c r="G7" s="89"/>
+      <c r="H7" s="89"/>
+      <c r="I7" s="90"/>
+      <c r="J7" s="88" t="s">
         <v>8</v>
       </c>
-      <c r="K7" s="99"/>
-      <c r="L7" s="99"/>
-      <c r="M7" s="99"/>
-      <c r="N7" s="101" t="s">
+      <c r="K7" s="89"/>
+      <c r="L7" s="89"/>
+      <c r="M7" s="89"/>
+      <c r="N7" s="82" t="s">
         <v>9</v>
       </c>
-      <c r="O7" s="102"/>
-      <c r="P7" s="103"/>
+      <c r="O7" s="83"/>
+      <c r="P7" s="84"/>
     </row>
     <row r="8" spans="1:16" ht="32.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="10"/>
@@ -2388,93 +2397,93 @@
       <c r="C8" s="11"/>
       <c r="D8" s="12"/>
       <c r="E8" s="13"/>
-      <c r="F8" s="104" t="s">
+      <c r="F8" s="91" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="105"/>
-      <c r="H8" s="105"/>
-      <c r="I8" s="106"/>
-      <c r="J8" s="104"/>
-      <c r="K8" s="105"/>
-      <c r="L8" s="105"/>
-      <c r="M8" s="105"/>
-      <c r="N8" s="104"/>
-      <c r="O8" s="105"/>
-      <c r="P8" s="107"/>
+      <c r="G8" s="92"/>
+      <c r="H8" s="92"/>
+      <c r="I8" s="93"/>
+      <c r="J8" s="91"/>
+      <c r="K8" s="92"/>
+      <c r="L8" s="92"/>
+      <c r="M8" s="92"/>
+      <c r="N8" s="91"/>
+      <c r="O8" s="92"/>
+      <c r="P8" s="94"/>
     </row>
     <row r="9" spans="1:16" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="90" t="s">
+      <c r="A9" s="98" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="82"/>
-      <c r="C9" s="83"/>
-      <c r="D9" s="75" t="s">
+      <c r="B9" s="99"/>
+      <c r="C9" s="100"/>
+      <c r="D9" s="107" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="78" t="s">
+      <c r="E9" s="110" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="95" t="s">
+      <c r="F9" s="113" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="78" t="s">
+      <c r="G9" s="110" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="75" t="s">
+      <c r="H9" s="107" t="s">
         <v>16</v>
       </c>
-      <c r="I9" s="75" t="s">
+      <c r="I9" s="107" t="s">
         <v>17</v>
       </c>
-      <c r="J9" s="78" t="s">
+      <c r="J9" s="110" t="s">
         <v>18</v>
       </c>
-      <c r="K9" s="75" t="s">
+      <c r="K9" s="107" t="s">
         <v>19</v>
       </c>
-      <c r="L9" s="75" t="s">
+      <c r="L9" s="107" t="s">
         <v>20</v>
       </c>
-      <c r="M9" s="81" t="s">
+      <c r="M9" s="116" t="s">
         <v>21</v>
       </c>
-      <c r="N9" s="82"/>
-      <c r="O9" s="83"/>
-      <c r="P9" s="87" t="s">
+      <c r="N9" s="99"/>
+      <c r="O9" s="100"/>
+      <c r="P9" s="95" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:16" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="91"/>
-      <c r="B10" s="85"/>
-      <c r="C10" s="86"/>
-      <c r="D10" s="76"/>
-      <c r="E10" s="79"/>
-      <c r="F10" s="96"/>
-      <c r="G10" s="79"/>
-      <c r="H10" s="76"/>
-      <c r="I10" s="76"/>
-      <c r="J10" s="79"/>
-      <c r="K10" s="76"/>
-      <c r="L10" s="76"/>
-      <c r="M10" s="84"/>
-      <c r="N10" s="85"/>
-      <c r="O10" s="86"/>
-      <c r="P10" s="88"/>
+      <c r="A10" s="101"/>
+      <c r="B10" s="102"/>
+      <c r="C10" s="103"/>
+      <c r="D10" s="108"/>
+      <c r="E10" s="111"/>
+      <c r="F10" s="114"/>
+      <c r="G10" s="111"/>
+      <c r="H10" s="108"/>
+      <c r="I10" s="108"/>
+      <c r="J10" s="111"/>
+      <c r="K10" s="108"/>
+      <c r="L10" s="108"/>
+      <c r="M10" s="117"/>
+      <c r="N10" s="102"/>
+      <c r="O10" s="103"/>
+      <c r="P10" s="96"/>
     </row>
     <row r="11" spans="1:16" s="14" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="92"/>
-      <c r="B11" s="93"/>
-      <c r="C11" s="94"/>
-      <c r="D11" s="77"/>
-      <c r="E11" s="80"/>
-      <c r="F11" s="97"/>
-      <c r="G11" s="80"/>
-      <c r="H11" s="77"/>
-      <c r="I11" s="77"/>
-      <c r="J11" s="80"/>
-      <c r="K11" s="77"/>
-      <c r="L11" s="77"/>
+      <c r="A11" s="104"/>
+      <c r="B11" s="105"/>
+      <c r="C11" s="106"/>
+      <c r="D11" s="109"/>
+      <c r="E11" s="112"/>
+      <c r="F11" s="115"/>
+      <c r="G11" s="112"/>
+      <c r="H11" s="109"/>
+      <c r="I11" s="109"/>
+      <c r="J11" s="112"/>
+      <c r="K11" s="109"/>
+      <c r="L11" s="109"/>
       <c r="M11" s="15" t="s">
         <v>23</v>
       </c>
@@ -2484,12 +2493,14 @@
       <c r="O11" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="P11" s="89"/>
+      <c r="P11" s="97"/>
     </row>
     <row r="12" spans="1:16" s="14" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="67"/>
-      <c r="B12" s="68"/>
-      <c r="C12" s="69"/>
+      <c r="A12" s="118" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="119"/>
+      <c r="C12" s="120"/>
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
       <c r="F12" s="17"/>
@@ -2506,7 +2517,9 @@
     </row>
     <row r="13" spans="1:16" s="14" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="20"/>
-      <c r="B13" s="21"/>
+      <c r="B13" s="21" t="s">
+        <v>42</v>
+      </c>
       <c r="C13" s="22"/>
       <c r="D13" s="23"/>
       <c r="E13" s="23"/>
@@ -2525,7 +2538,9 @@
     <row r="14" spans="1:16" s="14" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="20"/>
       <c r="B14" s="25"/>
-      <c r="C14" s="22"/>
+      <c r="C14" s="22" t="s">
+        <v>43</v>
+      </c>
       <c r="D14" s="26"/>
       <c r="E14" s="26"/>
       <c r="F14" s="27"/>
@@ -2668,8 +2683,8 @@
     </row>
     <row r="22" spans="1:16" s="14" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="41"/>
-      <c r="B22" s="70"/>
-      <c r="C22" s="71"/>
+      <c r="B22" s="121"/>
+      <c r="C22" s="122"/>
       <c r="D22" s="29"/>
       <c r="E22" s="26"/>
       <c r="F22" s="38"/>
@@ -3016,10 +3031,10 @@
     <row r="41" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A41" s="56"/>
       <c r="B41" s="56"/>
-      <c r="C41" s="127" t="s">
+      <c r="C41" s="126" t="s">
         <v>38</v>
       </c>
-      <c r="D41" s="126"/>
+      <c r="D41" s="127"/>
       <c r="E41" s="56"/>
       <c r="F41" s="56"/>
       <c r="G41" s="56"/>
@@ -3029,36 +3044,36 @@
       <c r="I41" s="129"/>
       <c r="J41" s="56"/>
       <c r="K41" s="56"/>
-      <c r="L41" s="127" t="s">
+      <c r="L41" s="126" t="s">
         <v>41</v>
       </c>
-      <c r="M41" s="127"/>
-      <c r="N41" s="127"/>
-      <c r="O41" s="127"/>
+      <c r="M41" s="126"/>
+      <c r="N41" s="126"/>
+      <c r="O41" s="126"/>
       <c r="P41" s="56"/>
     </row>
     <row r="42" spans="1:16" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A42" s="59"/>
       <c r="B42" s="59"/>
-      <c r="C42" s="72" t="s">
+      <c r="C42" s="123" t="s">
         <v>38</v>
       </c>
-      <c r="D42" s="72"/>
+      <c r="D42" s="123"/>
       <c r="E42" s="65"/>
       <c r="F42" s="65"/>
       <c r="G42" s="65"/>
-      <c r="H42" s="73" t="s">
+      <c r="H42" s="124" t="s">
         <v>39</v>
       </c>
-      <c r="I42" s="73"/>
+      <c r="I42" s="124"/>
       <c r="J42" s="65"/>
       <c r="K42" s="65"/>
-      <c r="L42" s="74" t="s">
+      <c r="L42" s="125" t="s">
         <v>40</v>
       </c>
-      <c r="M42" s="74"/>
-      <c r="N42" s="74"/>
-      <c r="O42" s="74"/>
+      <c r="M42" s="125"/>
+      <c r="N42" s="125"/>
+      <c r="O42" s="125"/>
       <c r="P42" s="59"/>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
@@ -3066,22 +3081,14 @@
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="J3:M3"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="F4:I6"/>
-    <mergeCell ref="J4:M4"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="J5:M5"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="J6:M6"/>
-    <mergeCell ref="N6:P6"/>
-    <mergeCell ref="F7:I7"/>
-    <mergeCell ref="J7:M7"/>
-    <mergeCell ref="N7:P7"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="J8:M8"/>
-    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="L42:O42"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="H41:I41"/>
+    <mergeCell ref="L41:O41"/>
     <mergeCell ref="P9:P11"/>
     <mergeCell ref="A9:C11"/>
     <mergeCell ref="D9:D11"/>
@@ -3094,14 +3101,22 @@
     <mergeCell ref="K9:K11"/>
     <mergeCell ref="L9:L11"/>
     <mergeCell ref="M9:O10"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="L42:O42"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="H41:I41"/>
-    <mergeCell ref="L41:O41"/>
+    <mergeCell ref="F7:I7"/>
+    <mergeCell ref="J7:M7"/>
+    <mergeCell ref="N7:P7"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="J8:M8"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="J3:M3"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="F4:I6"/>
+    <mergeCell ref="J4:M4"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="J5:M5"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="J6:M6"/>
+    <mergeCell ref="N6:P6"/>
   </mergeCells>
   <pageMargins left="0.23622047244094491" right="0.19685039370078741" top="0.23622047244094491" bottom="0.39370078740157483" header="0.11811023622047245" footer="0"/>
   <pageSetup paperSize="256" scale="60" orientation="landscape" horizontalDpi="4294967293" r:id="rId1"/>

</xml_diff>